<commit_message>
chapter 2 and 3 update
</commit_message>
<xml_diff>
--- a/Tese Tasks.xlsx
+++ b/Tese Tasks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10315"/>
   <workbookPr codeName="ThisWorkbook" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0a01f24622f98768/Ambiente de Trabalho/Oflat/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Desktop/Oflat/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:11_{8E0E5C28-86C1-4F47-8526-089017213898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FCE566F8-F41B-49F8-AFA6-DE8FBF1BF18C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="23260" windowHeight="13180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TASKS" sheetId="1" r:id="rId1"/>
@@ -260,7 +260,7 @@
     <cellStyle name="Done" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
-    <cellStyle name="Percent" xfId="4" builtinId="5" customBuiltin="1"/>
+    <cellStyle name="Per cent" xfId="4" builtinId="5" customBuiltin="1"/>
     <cellStyle name="Table Text" xfId="6" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
     <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
   </cellStyles>
@@ -372,10 +372,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -611,19 +607,19 @@
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:G22"/>
-  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="33" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="33" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
     <col min="2" max="2" width="104.6640625" customWidth="1"/>
-    <col min="3" max="3" width="19.77734375" customWidth="1"/>
-    <col min="4" max="4" width="16.44140625" customWidth="1"/>
-    <col min="5" max="5" width="18.77734375" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.5" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
     <col min="6" max="6" width="3" customWidth="1"/>
     <col min="7" max="7" width="90.6640625" customWidth="1"/>
-    <col min="8" max="8" width="2.44140625" customWidth="1"/>
+    <col min="8" max="8" width="2.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
         <v>16</v>
       </c>
@@ -633,7 +629,7 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
@@ -653,7 +649,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="9" t="s">
         <v>7</v>
       </c>
@@ -672,7 +668,7 @@
       </c>
       <c r="G3" s="7"/>
     </row>
-    <row r="4" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="7" t="s">
         <v>9</v>
       </c>
@@ -691,7 +687,7 @@
       </c>
       <c r="G4" s="7"/>
     </row>
-    <row r="5" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="7" t="s">
         <v>12</v>
       </c>
@@ -710,7 +706,7 @@
       </c>
       <c r="G5" s="7"/>
     </row>
-    <row r="6" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="7" t="s">
         <v>13</v>
       </c>
@@ -729,7 +725,7 @@
       </c>
       <c r="G6" s="7"/>
     </row>
-    <row r="7" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="7" t="s">
         <v>20</v>
       </c>
@@ -748,7 +744,7 @@
       </c>
       <c r="G7" s="7"/>
     </row>
-    <row r="8" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="7" t="s">
         <v>8</v>
       </c>
@@ -767,7 +763,7 @@
       </c>
       <c r="G8" s="7"/>
     </row>
-    <row r="9" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="7" t="s">
         <v>10</v>
       </c>
@@ -788,7 +784,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="7" t="s">
         <v>21</v>
       </c>
@@ -807,7 +803,7 @@
       </c>
       <c r="G10" s="7"/>
     </row>
-    <row r="11" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="7" t="s">
         <v>22</v>
       </c>
@@ -826,7 +822,7 @@
       </c>
       <c r="G11" s="7"/>
     </row>
-    <row r="12" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="7" t="s">
         <v>23</v>
       </c>
@@ -845,7 +841,7 @@
       </c>
       <c r="G12" s="7"/>
     </row>
-    <row r="13" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="7" t="s">
         <v>24</v>
       </c>
@@ -864,7 +860,7 @@
       </c>
       <c r="G13" s="7"/>
     </row>
-    <row r="14" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="7" t="s">
         <v>14</v>
       </c>
@@ -885,7 +881,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="7" t="s">
         <v>17</v>
       </c>
@@ -906,7 +902,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="7"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
@@ -916,7 +912,7 @@
       </c>
       <c r="G16" s="7"/>
     </row>
-    <row r="22" spans="2:2" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:2" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
         <v>19</v>
       </c>

</xml_diff>